<commit_message>
feat: add column headers to Excel files for user-friendliness
Changes:
- Added descriptive column headers to all Excel files
- Updated Python script to skip first row (skiprows=1)
- Headers help users understand what goes where
- Script still uses iloc (position-based) for simplicity

Excel files now have headers like:
- header: field, value
- experience: title, company, location, start_date, end_date, bullet_1, bullet_2...
- skills: category, skills
- education: degree, institution, location, start_year, end_year, detail_1...

Makes Excel editing much more intuitive!
</commit_message>
<xml_diff>
--- a/profiles/resume_data.xlsx
+++ b/profiles/resume_data.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="header" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="experience" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="education" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="skills" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="volunteering" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hobbies" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Certificates" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="header" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="experience" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="education" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="skills" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="volunteering" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Hobbies" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Certificates" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,13 +24,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +44,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -49,12 +52,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,52 +432,64 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>John Doe</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>+1 (555) 123-4567</t>
+          <t>John Doe</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>john.doe@email.com</t>
+          <t>+1 (555) 123-4567</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>john.doe@email.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>linkedin.com/in/johndoe</t>
         </is>
@@ -482,11 +506,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Brief professional summary highlighting your key expertise, experience, and value proposition. Focus on your core competencies and what makes you unique as a professional.</t>
         </is>
@@ -503,88 +534,130 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Senior Engineer</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>TechCorp</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>San Francisco, CA</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Led key initiatives resulting in measurable business impact and improved operational efficiency.</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Developed and implemented solutions that enhanced team productivity and project delivery.</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Collaborated with cross-functional teams to drive strategic objectives and innovation.</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>start_date</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>bullet_1</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>bullet_2</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>bullet_3</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Senior Engineer</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TechCorp</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Led key initiatives resulting in measurable business impact and improved operational efficiency.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Developed and implemented solutions that enhanced team productivity and project delivery.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Collaborated with cross-functional teams to drive strategic objectives and innovation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>StartupXYZ</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>2017</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Managed critical projects from conception to deployment with successful outcomes.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Built scalable systems and processes that improved organizational capabilities.</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Mentored team members and contributed to knowledge sharing initiatives.</t>
         </is>
@@ -601,41 +674,78 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>institution</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>start_year</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>end_year</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>detail_1</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>detail_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Bachelor of Science in Computer Science</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>University Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Boston, MA</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>2013</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>2017</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Focus on software engineering, algorithms, and data structures.</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Relevant coursework: Machine Learning, Database Systems, Web Development.</t>
         </is>
@@ -652,28 +762,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Programming &amp; Frameworks</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Python, JavaScript, React, Node.js, Django, Flask</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>skills</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Programming &amp; Frameworks</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Python, JavaScript, React, Node.js, Django, Flask</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Tools &amp; Technologies</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Git, Docker, AWS, PostgreSQL, MongoDB, CI/CD</t>
         </is>
@@ -690,21 +812,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>organization</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Tech Mentor</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Local Nonprofit Organization</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2021 -- Present</t>
         </is>
@@ -721,25 +860,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Gardening</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>hobby</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Playing Board Games</t>
+          <t>Gardening</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
+        <is>
+          <t>Playing Board Games</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Reading Science Fiction</t>
         </is>
@@ -756,28 +902,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Python Programming</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Python Programming A to Z by Coursera</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>certificate</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>details</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Python Programming</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Python Programming A to Z by Coursera</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Project Management</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Introduction to Project Management - PMI 2022</t>
         </is>

</xml_diff>